<commit_message>
Fix user reference in booking deletion event trigger, update booking import excel template to include Airline
</commit_message>
<xml_diff>
--- a/public/import_template.xlsx
+++ b/public/import_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10912"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daveroverts/code/sites/bmac/public/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nkevins/Workspace/bmac/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{350A604C-C307-1B42-970D-B497DA28A4A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20287FAB-F51E-8242-9A47-18F534BDD7D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="29040" windowHeight="15840" xr2:uid="{D04AF5E1-FD0B-423F-91F9-BDC72DF41FA8}"/>
+    <workbookView xWindow="6960" yWindow="5840" windowWidth="29040" windowHeight="15840" xr2:uid="{D04AF5E1-FD0B-423F-91F9-BDC72DF41FA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Call Sign</t>
   </si>
@@ -44,19 +44,22 @@
     <t>Destination</t>
   </si>
   <si>
+    <t>Aircraft Type</t>
+  </si>
+  <si>
+    <t>Route</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Airline</t>
+  </si>
+  <si>
+    <t>CTOT</t>
+  </si>
+  <si>
     <t>ETA</t>
-  </si>
-  <si>
-    <t>Aircraft Type</t>
-  </si>
-  <si>
-    <t>Route</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>CTOT</t>
   </si>
 </sst>
 </file>
@@ -112,7 +115,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -128,9 +131,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Kantoorthema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -168,7 +171,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -274,7 +277,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -416,7 +419,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -424,17 +427,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91403348-4099-4258-BDAA-3E7E76500E16}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.1640625" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -444,20 +448,23 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update import to include bay
</commit_message>
<xml_diff>
--- a/public/import_template.xlsx
+++ b/public/import_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nkevins/Workspace/bmac/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20287FAB-F51E-8242-9A47-18F534BDD7D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{125CD6FB-D375-A74B-9E6C-B27DB9024205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6960" yWindow="5840" windowWidth="29040" windowHeight="15840" xr2:uid="{D04AF5E1-FD0B-423F-91F9-BDC72DF41FA8}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Call Sign</t>
   </si>
@@ -60,6 +60,12 @@
   </si>
   <si>
     <t>ETA</t>
+  </si>
+  <si>
+    <t>Origin Bay</t>
+  </si>
+  <si>
+    <t>Destination Bay</t>
   </si>
 </sst>
 </file>
@@ -427,18 +433,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91403348-4099-4258-BDAA-3E7E76500E16}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.33203125" customWidth="1"/>
-    <col min="7" max="7" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.1640625" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="9" max="9" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -446,24 +454,30 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>